<commit_message>
Added invalid login and register
</commit_message>
<xml_diff>
--- a/data_provider/DataProvider.xlsx
+++ b/data_provider/DataProvider.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pytest_Automation_Project\Pytest_Automation_Project\data_provider\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{604AE1AA-0AFC-4A1A-98DB-7C97C9586151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA0438A-0D55-49E2-9533-0ADE7E7638F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3984" yWindow="1752" windowWidth="17280" windowHeight="9948" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3984" yWindow="1752" windowWidth="17280" windowHeight="9948" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginDataValid" sheetId="1" r:id="rId1"/>
+    <sheet name="loginDataInvalid" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
   <si>
     <t>email</t>
   </si>
@@ -37,6 +38,12 @@
   </si>
   <si>
     <t>testlogin</t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>rocket143@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -397,4 +404,33 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86FE512B-16B6-4250-AC75-D1CA861F7759}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{7B08D1EF-C470-4A90-80F4-CA979EF4DEF5}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
implement the excel file in registration checkout
</commit_message>
<xml_diff>
--- a/data_provider/DataProvider.xlsx
+++ b/data_provider/DataProvider.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pytest_Automation_Project\Pytest_Automation_Project\data_provider\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pytest_Automation_Project\data_provider\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{604AE1AA-0AFC-4A1A-98DB-7C97C9586151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3984" yWindow="1752" windowWidth="17280" windowHeight="9948" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3980" yWindow="1750" windowWidth="17280" windowHeight="9950" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="loginDataValid" sheetId="1" r:id="rId1"/>
+    <sheet name="Registeration" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
   <si>
     <t>email</t>
   </si>
@@ -37,12 +37,75 @@
   </si>
   <si>
     <t>testlogin</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Telephone</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>ConfirmPassword</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Address1</t>
+  </si>
+  <si>
+    <t>Address2</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Doe</t>
+  </si>
+  <si>
+    <t>johndoe12345@gmail.com</t>
+  </si>
+  <si>
+    <t>Test@1234</t>
+  </si>
+  <si>
+    <t>smartcliff</t>
+  </si>
+  <si>
+    <t>123 Test street</t>
+  </si>
+  <si>
+    <t>Apt 4B</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>New york</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -371,11 +434,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -383,7 +446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -393,7 +456,112 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{B720FABE-1E88-4423-A5BD-692A31F09060}"/>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.6328125" customWidth="1"/>
+    <col min="2" max="2" width="12.36328125" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="4" max="4" width="15.26953125" customWidth="1"/>
+    <col min="5" max="5" width="14.1796875" customWidth="1"/>
+    <col min="6" max="6" width="16.453125" customWidth="1"/>
+    <col min="7" max="7" width="12.36328125" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="16.1796875" customWidth="1"/>
+    <col min="10" max="10" width="13.36328125" customWidth="1"/>
+    <col min="11" max="11" width="12.81640625" customWidth="1"/>
+    <col min="12" max="12" width="11.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2">
+        <v>9698618786</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1"/>
+    <hyperlink ref="E2" r:id="rId2"/>
+    <hyperlink ref="F2" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Addreviewpage and excel
</commit_message>
<xml_diff>
--- a/data_provider/DataProvider.xlsx
+++ b/data_provider/DataProvider.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pytest_Automation_Project\data_provider\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{310B53C5-054A-4FE6-9A8C-9DDF8F351C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7180" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="10800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginDataValid" sheetId="1" r:id="rId1"/>
     <sheet name="loginDataInvalid" sheetId="2" r:id="rId2"/>
     <sheet name="Registration" sheetId="3" r:id="rId3"/>
+    <sheet name="AddReview-valid" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -26,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
   <si>
     <t>email</t>
   </si>
@@ -131,11 +133,32 @@
   <si>
     <t>testuserjohn@gmail.com</t>
   </si>
+  <si>
+    <t>rating</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>feedback</t>
+  </si>
+  <si>
+    <t>expectedMessage</t>
+  </si>
+  <si>
+    <t>Joshi</t>
+  </si>
+  <si>
+    <t>The product is really good to use and easy to maintain.Also durable one</t>
+  </si>
+  <si>
+    <t>Thank you for your review. It has been submitted to the webmaster for approval.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -473,11 +496,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -485,7 +508,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -495,22 +518,22 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="8.7265625" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -518,7 +541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
@@ -528,33 +551,33 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" customWidth="1"/>
-    <col min="2" max="2" width="20.6328125" customWidth="1"/>
-    <col min="3" max="3" width="21.6328125" customWidth="1"/>
-    <col min="4" max="4" width="16.453125" customWidth="1"/>
-    <col min="5" max="5" width="15.36328125" customWidth="1"/>
-    <col min="6" max="6" width="16.36328125" customWidth="1"/>
-    <col min="7" max="7" width="12.81640625" customWidth="1"/>
-    <col min="8" max="8" width="14.7265625" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="21.5703125" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
-    <col min="10" max="10" width="16.54296875" customWidth="1"/>
-    <col min="11" max="11" width="20.453125" customWidth="1"/>
-    <col min="12" max="12" width="13.6328125" customWidth="1"/>
-    <col min="13" max="13" width="13.1796875" customWidth="1"/>
+    <col min="10" max="10" width="16.5703125" customWidth="1"/>
+    <col min="11" max="11" width="20.42578125" customWidth="1"/>
+    <col min="12" max="12" width="13.5703125" customWidth="1"/>
+    <col min="13" max="13" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>17</v>
       </c>
@@ -595,7 +618,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -638,11 +661,54 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1"/>
-    <hyperlink ref="E2" r:id="rId2"/>
-    <hyperlink ref="C2" r:id="rId3"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="E2" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
+    <hyperlink ref="C2" r:id="rId3" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B62B96E-9D26-49BA-895B-7AF9559CF189}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="22.42578125" customWidth="1"/>
+    <col min="3" max="3" width="74.42578125" customWidth="1"/>
+    <col min="4" max="4" width="104" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added the test Compare test cases
</commit_message>
<xml_diff>
--- a/data_provider/DataProvider.xlsx
+++ b/data_provider/DataProvider.xlsx
@@ -5,17 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pytest_Automation_Project\Pytest_Automation_Project\data_provider\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Pytest_Automation\data_provider\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC2846CE-8706-40B2-8750-D23C65DFDA99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C07A007-F904-420F-A1B3-7A79627E0F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4332" yWindow="2100" windowWidth="17280" windowHeight="9948" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginDataValid" sheetId="1" r:id="rId1"/>
     <sheet name="loginDataInvalid" sheetId="2" r:id="rId2"/>
-    <sheet name="Registration" sheetId="3" r:id="rId3"/>
+    <sheet name="EnquiryData" sheetId="4" r:id="rId3"/>
+    <sheet name="Registration" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
   <si>
     <t>email</t>
   </si>
@@ -131,6 +132,27 @@
   </si>
   <si>
     <t>camera143@gmail.com</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>subject</t>
+  </si>
+  <si>
+    <t>Message</t>
+  </si>
+  <si>
+    <t>Tamil Kumar</t>
+  </si>
+  <si>
+    <t>abc@gmail.com</t>
+  </si>
+  <si>
+    <t>Product Damage</t>
+  </si>
+  <si>
+    <t>When I recived the product it is damaged</t>
   </si>
 </sst>
 </file>
@@ -536,6 +558,47 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7CE0A72-D28D-4946-9D4D-84D0C7BA7189}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{AEA6EBB8-B108-4DA3-AA5F-0ACD45BB6756}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Added invalid review with rating only
</commit_message>
<xml_diff>
--- a/data_provider/DataProvider.xlsx
+++ b/data_provider/DataProvider.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pytest_Automation_Project\data_provider\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4419CE97-9239-4921-96B0-15BD2288ED6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87941601-6787-469C-BEAC-385A90885373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginDataValid" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="EnquiryData" sheetId="4" r:id="rId3"/>
     <sheet name="Registration" sheetId="3" r:id="rId4"/>
     <sheet name="AddReview-valid" sheetId="5" r:id="rId5"/>
+    <sheet name="AddReview-rating" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
   <si>
     <t>email</t>
   </si>
@@ -175,6 +176,9 @@
   </si>
   <si>
     <t>Thank you for your review. It has been submitted to the webmaster for approval.</t>
+  </si>
+  <si>
+    <t>Warning: Review Text must be between 25 and 1000 characters!</t>
   </si>
 </sst>
 </file>
@@ -773,4 +777,33 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{521EE4DF-EDD3-4FBB-A2DC-241DA6F48EC8}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="82" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Changed The Excel Data for invalid Register
</commit_message>
<xml_diff>
--- a/data_provider/DataProvider.xlsx
+++ b/data_provider/DataProvider.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pytest_Automation_Project\Pytest_Automation_Project\data_provider\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC2846CE-8706-40B2-8750-D23C65DFDA99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A2B46A4-C425-43C6-90FB-E9C61E5E1266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4332" yWindow="2100" windowWidth="17280" windowHeight="9948" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -130,7 +130,7 @@
     <t>testuserjohn@gmail.com</t>
   </si>
   <si>
-    <t>camera143@gmail.com</t>
+    <t>GameOfThrones@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Completed addreview feature and added AddOns
</commit_message>
<xml_diff>
--- a/data_provider/DataProvider.xlsx
+++ b/data_provider/DataProvider.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pytest_Automation_Project\data_provider\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87941601-6787-469C-BEAC-385A90885373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D5D86F7-ED8B-4104-8CD8-41D859024EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginDataValid" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,9 @@
     <sheet name="Registration" sheetId="3" r:id="rId4"/>
     <sheet name="AddReview-valid" sheetId="5" r:id="rId5"/>
     <sheet name="AddReview-rating" sheetId="6" r:id="rId6"/>
+    <sheet name="AddReview-withoutname" sheetId="7" r:id="rId7"/>
+    <sheet name="AddReview-withoutfeedback" sheetId="8" r:id="rId8"/>
+    <sheet name="AddReview-withoutrating" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -30,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="46">
   <si>
     <t>email</t>
   </si>
@@ -179,6 +182,15 @@
   </si>
   <si>
     <t>Warning: Review Text must be between 25 and 1000 characters!</t>
+  </si>
+  <si>
+    <t>Warning: Review Name must be between 3 and 25 characters!</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Warning: Please select a review rating!</t>
   </si>
 </sst>
 </file>
@@ -806,4 +818,119 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C7F3E0E-94E6-417E-BB92-5EBB9A3A7B61}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="91.85546875" customWidth="1"/>
+    <col min="4" max="4" width="78.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BFA7B0A-6BA3-4F04-AAE5-DD461429D9F6}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="76" customWidth="1"/>
+    <col min="4" max="4" width="109.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AA6D1D9-307D-41A6-B231-052C850287FA}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="90.140625" customWidth="1"/>
+    <col min="3" max="3" width="82.42578125" customWidth="1"/>
+    <col min="4" max="4" width="85.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>